<commit_message>
Site guncellemesi - 23.09.2026 18:47
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/yükselis-hacim.xlsx
+++ b/app/borsa/gosterge-taramalari/data/yükselis-hacim.xlsx
@@ -26,46 +26,13 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>AHGAZ</x:t>
+    <x:t>XU100</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
   </x:si>
   <x:si>
     <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAHKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KCHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMD</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -416,7 +383,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C8"/>
+  <x:dimension ref="A1:C1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -428,83 +395,6 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3">
-      <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -521,7 +411,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C6"/>
+  <x:dimension ref="A1:C2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -537,56 +427,12 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 25.09.2026 18:31
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/yükselis-hacim.xlsx
+++ b/app/borsa/gosterge-taramalari/data/yükselis-hacim.xlsx
@@ -26,49 +26,55 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>BAHKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETILR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKYMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRMET</x:t>
+  </x:si>
+  <x:si>
     <x:t>AHGAZ</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
     <x:t>ISDMR</x:t>
   </x:si>
   <x:si>
+    <x:t>KRDMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORGE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYGYO</x:t>
+  </x:si>
+  <x:si>
     <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRMET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUPRS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -419,7 +425,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C6"/>
+  <x:dimension ref="A1:C7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -485,6 +491,17 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -502,7 +519,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C9"/>
+  <x:dimension ref="A1:C10"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -518,7 +535,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -529,7 +546,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -540,7 +557,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -551,7 +568,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -562,7 +579,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -573,7 +590,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -584,7 +601,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -595,12 +612,23 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:3">
+      <x:c r="A10" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 28.09.2026 18:22
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/yükselis-hacim.xlsx
+++ b/app/borsa/gosterge-taramalari/data/yükselis-hacim.xlsx
@@ -26,52 +26,43 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>ETILR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKYMD</x:t>
+  </x:si>
+  <x:si>
     <x:t>BAHKM</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRMET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
+    <x:t>BIMAS</x:t>
   </x:si>
   <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
+    <x:t>FLAP</x:t>
   </x:si>
   <x:si>
     <x:t>KRDMD</x:t>
   </x:si>
   <x:si>
-    <x:t>ORGE</x:t>
-  </x:si>
-  <x:si>
     <x:t>RYGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYSAS</x:t>
   </x:si>
   <x:si>
     <x:t>TKFEN</x:t>
@@ -425,7 +416,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C7"/>
+  <x:dimension ref="A1:C5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -480,28 +471,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -519,7 +488,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C10"/>
+  <x:dimension ref="A1:C9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -535,7 +504,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -546,7 +515,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -557,7 +526,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -568,7 +537,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -579,7 +548,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -590,7 +559,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -601,7 +570,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -612,23 +581,12 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:3">
-      <x:c r="A10" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>